<commit_message>
doc(work logs) : fixing the problem
Last time I lost some of my changes, this file contains all of my logs
</commit_message>
<xml_diff>
--- a/T-CraftMeUp_JonathanJunod.xlsx
+++ b/T-CraftMeUp_JonathanJunod.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pe40boh\Documents\GitHub\Craft-Me-Up\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:11_{49C3D4D1-FA8C-4A30-8C9B-417FD5D42074}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9576ADC9-0FD6-46F1-AA62-C7E1494D755E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-75" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
     <sheet name="Restrictions" sheetId="19" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$G$54</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$G$48</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="58">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -186,6 +186,45 @@
   </si>
   <si>
     <t>https://eduvaud-my.sharepoint.com/:u:/r/personal/pb62kjx_eduvaud_ch/_layouts/15/Doc.aspx?sourcedoc=%7B5BF0A89E-E3A6-4CD4-BA7E-BFDC17A68BD3%7D&amp;file=P_CraftMeUp_ClassDiagram.vsdx&amp;fromShare=true&amp;action=default&amp;mobileredirect=true</t>
+  </si>
+  <si>
+    <t>Creating a new version of the classes diagram</t>
+  </si>
+  <si>
+    <t>Debating about the code optimization</t>
+  </si>
+  <si>
+    <t>Debating</t>
+  </si>
+  <si>
+    <t>Github project</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adding a kanban to github </t>
+  </si>
+  <si>
+    <t>Read and complete the CdC written by Neo</t>
+  </si>
+  <si>
+    <t>CdC</t>
+  </si>
+  <si>
+    <t>Coding</t>
+  </si>
+  <si>
+    <t>Correcting the obstacle class</t>
+  </si>
+  <si>
+    <t>https://github.com/users/Jonathan150408/projects/4/views/1</t>
+  </si>
+  <si>
+    <t>Git-problem</t>
+  </si>
+  <si>
+    <t>Solving a problem with the github project issues</t>
+  </si>
+  <si>
+    <t>https://github.com/users/Jonathan150408/projects/6/views/1</t>
   </si>
 </sst>
 </file>
@@ -397,7 +436,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -480,6 +519,31 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="20" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -488,44 +552,23 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -927,7 +970,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" style="1" customWidth="1"/>
@@ -945,65 +988,65 @@
       <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="32" t="s">
+      <c r="B1" s="27" t="s">
         <v>36</v>
       </c>
-      <c r="C1" s="33"/>
-      <c r="D1" s="30" t="s">
+      <c r="C1" s="29"/>
+      <c r="D1" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="31"/>
-      <c r="F1" s="28" t="s">
+      <c r="E1" s="36"/>
+      <c r="F1" s="33" t="s">
         <v>37</v>
       </c>
-      <c r="G1" s="29"/>
+      <c r="G1" s="34"/>
     </row>
     <row r="2" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="32" t="s">
+      <c r="B2" s="27" t="s">
         <v>35</v>
       </c>
-      <c r="C2" s="33"/>
-      <c r="D2" s="30" t="s">
+      <c r="C2" s="29"/>
+      <c r="D2" s="35" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="31"/>
-      <c r="F2" s="28" t="s">
+      <c r="E2" s="36"/>
+      <c r="F2" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="29"/>
+      <c r="G2" s="34"/>
     </row>
     <row r="3" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="32" t="s">
+      <c r="B3" s="27" t="s">
         <v>34</v>
       </c>
-      <c r="C3" s="33"/>
-      <c r="D3" s="30" t="s">
+      <c r="C3" s="29"/>
+      <c r="D3" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="31"/>
-      <c r="F3" s="32" t="s">
+      <c r="E3" s="36"/>
+      <c r="F3" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="G3" s="33"/>
+      <c r="G3" s="29"/>
     </row>
     <row r="4" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="32" t="s">
+      <c r="B4" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="C4" s="36"/>
-      <c r="D4" s="36"/>
-      <c r="E4" s="36"/>
-      <c r="F4" s="36"/>
-      <c r="G4" s="33"/>
+      <c r="C4" s="28"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="28"/>
+      <c r="G4" s="29"/>
     </row>
     <row r="5" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1032,7 +1075,7 @@
       <c r="A6" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="23">
+      <c r="B6" s="30">
         <v>45964</v>
       </c>
       <c r="C6" s="5">
@@ -1044,7 +1087,7 @@
       <c r="E6" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="F6" s="37">
+      <c r="F6" s="24">
         <v>0.59027777777777779</v>
       </c>
       <c r="G6" s="19" t="s">
@@ -1055,7 +1098,7 @@
       <c r="A7" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="B7" s="24"/>
+      <c r="B7" s="31"/>
       <c r="C7" s="7">
         <v>35</v>
       </c>
@@ -1065,16 +1108,16 @@
       <c r="E7" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="F7" s="37">
+      <c r="F7" s="24">
         <v>0.61458333333333337</v>
       </c>
       <c r="G7" s="19"/>
     </row>
-    <row r="8" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="B8" s="24"/>
+      <c r="B8" s="31"/>
       <c r="C8" s="7">
         <v>45</v>
       </c>
@@ -1084,29 +1127,50 @@
       <c r="E8" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="F8" s="37">
+      <c r="F8" s="24">
         <v>0.65625</v>
       </c>
       <c r="G8" s="19" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="6"/>
-      <c r="B9" s="24"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="19"/>
+    <row r="9" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="25">
+        <f>SUM(C6:C8)</f>
+        <v>110</v>
+      </c>
+      <c r="E9" s="25"/>
+      <c r="F9" s="25"/>
+      <c r="G9" s="26"/>
     </row>
     <row r="10" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="9"/>
-      <c r="B10" s="25"/>
-      <c r="C10" s="9"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="7"/>
+      <c r="A10" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" s="23">
+        <v>45970</v>
+      </c>
+      <c r="C10" s="5">
+        <v>30</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="24">
+        <v>0.68055555555555547</v>
+      </c>
       <c r="G10" s="19"/>
     </row>
     <row r="11" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1114,85 +1178,141 @@
         <v>12</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C11" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="34">
-        <f>SUM(C6:C10)</f>
-        <v>110</v>
-      </c>
-      <c r="E11" s="34"/>
-      <c r="F11" s="34"/>
-      <c r="G11" s="35"/>
+      <c r="D11" s="25">
+        <f>SUM(C10:C10)</f>
+        <v>30</v>
+      </c>
+      <c r="E11" s="25"/>
+      <c r="F11" s="25"/>
+      <c r="G11" s="26"/>
     </row>
     <row r="12" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="4"/>
-      <c r="B12" s="23"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="22"/>
+      <c r="A12" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" s="30">
+        <v>45971</v>
+      </c>
+      <c r="C12" s="5">
+        <v>45</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="24">
+        <v>0.57986111111111105</v>
+      </c>
       <c r="G12" s="19"/>
     </row>
     <row r="13" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="6"/>
-      <c r="B13" s="24"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="22"/>
-      <c r="G13" s="19"/>
+      <c r="A13" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B13" s="31"/>
+      <c r="C13" s="7">
+        <v>5</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F13" s="24">
+        <v>0.58680555555555558</v>
+      </c>
+      <c r="G13" s="19" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="14" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="6"/>
-      <c r="B14" s="24"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="7"/>
+      <c r="A14" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B14" s="31"/>
+      <c r="C14" s="7">
+        <v>10</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F14" s="24">
+        <v>0.59375</v>
+      </c>
       <c r="G14" s="19"/>
     </row>
     <row r="15" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="6"/>
-      <c r="B15" s="24"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="7"/>
+      <c r="A15" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B15" s="31"/>
+      <c r="C15" s="7">
+        <v>50</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F15" s="24">
+        <v>0.65625</v>
+      </c>
       <c r="G15" s="19"/>
     </row>
     <row r="16" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="9"/>
-      <c r="B16" s="25"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="19"/>
+      <c r="A16" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B16" s="32"/>
+      <c r="C16" s="9">
+        <v>25</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="F16" s="24">
+        <v>0.61458333333333337</v>
+      </c>
+      <c r="G16" s="19" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="17" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
         <v>12</v>
       </c>
       <c r="B17" s="17" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C17" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="D17" s="34">
+      <c r="D17" s="25">
         <f>SUM(C12:C16)</f>
-        <v>0</v>
-      </c>
-      <c r="E17" s="34"/>
-      <c r="F17" s="34"/>
-      <c r="G17" s="35"/>
+        <v>135</v>
+      </c>
+      <c r="E17" s="25"/>
+      <c r="F17" s="25"/>
+      <c r="G17" s="26"/>
     </row>
     <row r="18" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4"/>
-      <c r="B18" s="23"/>
+      <c r="B18" s="30"/>
       <c r="C18" s="5"/>
       <c r="D18" s="8"/>
       <c r="E18" s="8"/>
@@ -1201,7 +1321,7 @@
     </row>
     <row r="19" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6"/>
-      <c r="B19" s="24"/>
+      <c r="B19" s="31"/>
       <c r="C19" s="7"/>
       <c r="D19" s="8"/>
       <c r="E19" s="8"/>
@@ -1210,7 +1330,7 @@
     </row>
     <row r="20" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="6"/>
-      <c r="B20" s="24"/>
+      <c r="B20" s="31"/>
       <c r="C20" s="7"/>
       <c r="D20" s="8"/>
       <c r="E20" s="8"/>
@@ -1219,7 +1339,7 @@
     </row>
     <row r="21" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6"/>
-      <c r="B21" s="24"/>
+      <c r="B21" s="31"/>
       <c r="C21" s="7"/>
       <c r="D21" s="8"/>
       <c r="E21" s="8"/>
@@ -1228,7 +1348,7 @@
     </row>
     <row r="22" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="9"/>
-      <c r="B22" s="25"/>
+      <c r="B22" s="32"/>
       <c r="C22" s="9"/>
       <c r="D22" s="8"/>
       <c r="E22" s="10"/>
@@ -1240,22 +1360,22 @@
         <v>12</v>
       </c>
       <c r="B23" s="17" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C23" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="D23" s="34">
+      <c r="D23" s="25">
         <f>SUM(C18:C22)</f>
         <v>0</v>
       </c>
-      <c r="E23" s="34"/>
-      <c r="F23" s="34"/>
-      <c r="G23" s="35"/>
+      <c r="E23" s="25"/>
+      <c r="F23" s="25"/>
+      <c r="G23" s="26"/>
     </row>
     <row r="24" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4"/>
-      <c r="B24" s="23"/>
+      <c r="B24" s="30"/>
       <c r="C24" s="5"/>
       <c r="D24" s="8"/>
       <c r="E24" s="8"/>
@@ -1264,7 +1384,7 @@
     </row>
     <row r="25" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="6"/>
-      <c r="B25" s="24"/>
+      <c r="B25" s="31"/>
       <c r="C25" s="7"/>
       <c r="D25" s="8"/>
       <c r="E25" s="8"/>
@@ -1273,7 +1393,7 @@
     </row>
     <row r="26" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="6"/>
-      <c r="B26" s="24"/>
+      <c r="B26" s="31"/>
       <c r="C26" s="7"/>
       <c r="D26" s="8"/>
       <c r="E26" s="8"/>
@@ -1282,7 +1402,7 @@
     </row>
     <row r="27" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="6"/>
-      <c r="B27" s="24"/>
+      <c r="B27" s="31"/>
       <c r="C27" s="7"/>
       <c r="D27" s="8"/>
       <c r="E27" s="8"/>
@@ -1291,7 +1411,7 @@
     </row>
     <row r="28" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="9"/>
-      <c r="B28" s="25"/>
+      <c r="B28" s="32"/>
       <c r="C28" s="9"/>
       <c r="D28" s="8"/>
       <c r="E28" s="10"/>
@@ -1303,22 +1423,22 @@
         <v>12</v>
       </c>
       <c r="B29" s="17" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C29" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="D29" s="34">
+      <c r="D29" s="25">
         <f>SUM(C24:C28)</f>
         <v>0</v>
       </c>
-      <c r="E29" s="34"/>
-      <c r="F29" s="34"/>
-      <c r="G29" s="35"/>
+      <c r="E29" s="25"/>
+      <c r="F29" s="25"/>
+      <c r="G29" s="26"/>
     </row>
     <row r="30" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="4"/>
-      <c r="B30" s="23"/>
+      <c r="B30" s="30"/>
       <c r="C30" s="5"/>
       <c r="D30" s="8"/>
       <c r="E30" s="8"/>
@@ -1327,7 +1447,7 @@
     </row>
     <row r="31" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="6"/>
-      <c r="B31" s="24"/>
+      <c r="B31" s="31"/>
       <c r="C31" s="7"/>
       <c r="D31" s="8"/>
       <c r="E31" s="8"/>
@@ -1336,7 +1456,7 @@
     </row>
     <row r="32" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="6"/>
-      <c r="B32" s="24"/>
+      <c r="B32" s="31"/>
       <c r="C32" s="7"/>
       <c r="D32" s="8"/>
       <c r="E32" s="8"/>
@@ -1345,7 +1465,7 @@
     </row>
     <row r="33" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="6"/>
-      <c r="B33" s="24"/>
+      <c r="B33" s="31"/>
       <c r="C33" s="7"/>
       <c r="D33" s="8"/>
       <c r="E33" s="8"/>
@@ -1354,7 +1474,7 @@
     </row>
     <row r="34" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="9"/>
-      <c r="B34" s="25"/>
+      <c r="B34" s="32"/>
       <c r="C34" s="9"/>
       <c r="D34" s="8"/>
       <c r="E34" s="10"/>
@@ -1366,22 +1486,22 @@
         <v>12</v>
       </c>
       <c r="B35" s="17" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C35" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="D35" s="34">
+      <c r="D35" s="25">
         <f>SUM(C30:C34)</f>
         <v>0</v>
       </c>
-      <c r="E35" s="34"/>
-      <c r="F35" s="34"/>
-      <c r="G35" s="35"/>
+      <c r="E35" s="25"/>
+      <c r="F35" s="25"/>
+      <c r="G35" s="26"/>
     </row>
     <row r="36" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="4"/>
-      <c r="B36" s="23"/>
+      <c r="B36" s="30"/>
       <c r="C36" s="5"/>
       <c r="D36" s="8"/>
       <c r="E36" s="8"/>
@@ -1390,7 +1510,7 @@
     </row>
     <row r="37" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="6"/>
-      <c r="B37" s="24"/>
+      <c r="B37" s="31"/>
       <c r="C37" s="7"/>
       <c r="D37" s="8"/>
       <c r="E37" s="8"/>
@@ -1399,7 +1519,7 @@
     </row>
     <row r="38" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="6"/>
-      <c r="B38" s="24"/>
+      <c r="B38" s="31"/>
       <c r="C38" s="7"/>
       <c r="D38" s="8"/>
       <c r="E38" s="8"/>
@@ -1408,7 +1528,7 @@
     </row>
     <row r="39" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="6"/>
-      <c r="B39" s="24"/>
+      <c r="B39" s="31"/>
       <c r="C39" s="7"/>
       <c r="D39" s="8"/>
       <c r="E39" s="8"/>
@@ -1417,7 +1537,7 @@
     </row>
     <row r="40" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="9"/>
-      <c r="B40" s="25"/>
+      <c r="B40" s="32"/>
       <c r="C40" s="9"/>
       <c r="D40" s="8"/>
       <c r="E40" s="10"/>
@@ -1429,22 +1549,22 @@
         <v>12</v>
       </c>
       <c r="B41" s="17" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C41" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="D41" s="34">
+      <c r="D41" s="25">
         <f>SUM(C36:C40)</f>
         <v>0</v>
       </c>
-      <c r="E41" s="34"/>
-      <c r="F41" s="34"/>
-      <c r="G41" s="35"/>
+      <c r="E41" s="25"/>
+      <c r="F41" s="25"/>
+      <c r="G41" s="26"/>
     </row>
     <row r="42" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="4"/>
-      <c r="B42" s="23"/>
+      <c r="B42" s="30"/>
       <c r="C42" s="5"/>
       <c r="D42" s="8"/>
       <c r="E42" s="8"/>
@@ -1453,7 +1573,7 @@
     </row>
     <row r="43" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="6"/>
-      <c r="B43" s="24"/>
+      <c r="B43" s="31"/>
       <c r="C43" s="7"/>
       <c r="D43" s="8"/>
       <c r="E43" s="8"/>
@@ -1462,7 +1582,7 @@
     </row>
     <row r="44" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="6"/>
-      <c r="B44" s="24"/>
+      <c r="B44" s="31"/>
       <c r="C44" s="7"/>
       <c r="D44" s="8"/>
       <c r="E44" s="8"/>
@@ -1471,7 +1591,7 @@
     </row>
     <row r="45" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="6"/>
-      <c r="B45" s="24"/>
+      <c r="B45" s="31"/>
       <c r="C45" s="7"/>
       <c r="D45" s="8"/>
       <c r="E45" s="8"/>
@@ -1480,7 +1600,7 @@
     </row>
     <row r="46" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="9"/>
-      <c r="B46" s="25"/>
+      <c r="B46" s="32"/>
       <c r="C46" s="9"/>
       <c r="D46" s="8"/>
       <c r="E46" s="10"/>
@@ -1492,118 +1612,49 @@
         <v>12</v>
       </c>
       <c r="B47" s="17" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C47" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="D47" s="34">
+      <c r="D47" s="25">
         <f>SUM(C42:C46)</f>
         <v>0</v>
       </c>
-      <c r="E47" s="34"/>
-      <c r="F47" s="34"/>
-      <c r="G47" s="35"/>
-    </row>
-    <row r="48" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="4"/>
-      <c r="B48" s="23"/>
-      <c r="C48" s="5"/>
-      <c r="D48" s="8"/>
-      <c r="E48" s="8"/>
-      <c r="F48" s="22"/>
-      <c r="G48" s="19"/>
-    </row>
-    <row r="49" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="6"/>
-      <c r="B49" s="24"/>
-      <c r="C49" s="7"/>
-      <c r="D49" s="8"/>
-      <c r="E49" s="8"/>
-      <c r="F49" s="22"/>
-      <c r="G49" s="19"/>
-    </row>
-    <row r="50" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="6"/>
-      <c r="B50" s="24"/>
-      <c r="C50" s="7"/>
-      <c r="D50" s="8"/>
-      <c r="E50" s="8"/>
-      <c r="F50" s="7"/>
-      <c r="G50" s="19"/>
-    </row>
-    <row r="51" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="6"/>
-      <c r="B51" s="24"/>
-      <c r="C51" s="7"/>
-      <c r="D51" s="8"/>
-      <c r="E51" s="8"/>
-      <c r="F51" s="7"/>
-      <c r="G51" s="19"/>
-    </row>
-    <row r="52" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="9"/>
-      <c r="B52" s="25"/>
-      <c r="C52" s="9"/>
-      <c r="D52" s="8"/>
-      <c r="E52" s="10"/>
-      <c r="F52" s="7"/>
-      <c r="G52" s="19"/>
-    </row>
-    <row r="53" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B53" s="17" t="s">
-        <v>26</v>
-      </c>
-      <c r="C53" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="D53" s="34">
-        <f>SUM(C48:C52)</f>
-        <v>0</v>
-      </c>
-      <c r="E53" s="34"/>
-      <c r="F53" s="34"/>
-      <c r="G53" s="35"/>
-    </row>
-    <row r="54" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="26" t="s">
+      <c r="E47" s="25"/>
+      <c r="F47" s="25"/>
+      <c r="G47" s="26"/>
+    </row>
+    <row r="48" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="B54" s="27"/>
-      <c r="C54" s="12">
-        <f>MROUND(SUM(C6:C53) /60,0.2)</f>
-        <v>1.8</v>
-      </c>
-      <c r="D54" s="13"/>
-      <c r="E54" s="18"/>
-      <c r="F54" s="20"/>
-      <c r="G54" s="14"/>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" s="15" t="s">
+      <c r="B48" s="38"/>
+      <c r="C48" s="12">
+        <f>MROUND(SUM(C6:C47) /60,0.2)</f>
+        <v>4.6000000000000005</v>
+      </c>
+      <c r="D48" s="13"/>
+      <c r="E48" s="18"/>
+      <c r="F48" s="20"/>
+      <c r="G48" s="14"/>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" s="15" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" s="15"/>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" s="15"/>
     </row>
   </sheetData>
-  <mergeCells count="27">
-    <mergeCell ref="D29:G29"/>
-    <mergeCell ref="D35:G35"/>
-    <mergeCell ref="D41:G41"/>
-    <mergeCell ref="D47:G47"/>
-    <mergeCell ref="D53:G53"/>
-    <mergeCell ref="D11:G11"/>
-    <mergeCell ref="D17:G17"/>
-    <mergeCell ref="D23:G23"/>
-    <mergeCell ref="B4:G4"/>
-    <mergeCell ref="B6:B10"/>
-    <mergeCell ref="B12:B16"/>
+  <mergeCells count="26">
     <mergeCell ref="B18:B22"/>
+    <mergeCell ref="B24:B28"/>
+    <mergeCell ref="B30:B34"/>
+    <mergeCell ref="A48:B48"/>
+    <mergeCell ref="B36:B40"/>
+    <mergeCell ref="B42:B46"/>
     <mergeCell ref="F1:G1"/>
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="D2:E2"/>
@@ -1613,18 +1664,23 @@
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="F3:G3"/>
-    <mergeCell ref="B24:B28"/>
-    <mergeCell ref="B30:B34"/>
-    <mergeCell ref="B36:B40"/>
-    <mergeCell ref="A54:B54"/>
-    <mergeCell ref="B42:B46"/>
-    <mergeCell ref="B48:B52"/>
+    <mergeCell ref="D9:G9"/>
+    <mergeCell ref="D11:G11"/>
+    <mergeCell ref="D17:G17"/>
+    <mergeCell ref="B4:G4"/>
+    <mergeCell ref="B6:B8"/>
+    <mergeCell ref="B12:B16"/>
+    <mergeCell ref="D23:G23"/>
+    <mergeCell ref="D29:G29"/>
+    <mergeCell ref="D35:G35"/>
+    <mergeCell ref="D41:G41"/>
+    <mergeCell ref="D47:G47"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C48:C52 C36:C40 C42:C46 C18:C22 B6 C12:C16 C24:C28 C30:C34 C6:C10" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C42:C46 C30:C34 C36:C40 C12:C16 B6 C10 C18:C22 C24:C28 C6:C8" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B12:B16 B18:B22 B24:B28 B30:B34 B36:B40 B42:B46 B48:B52" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B10 B12:B16 B18:B22 B24:B28 B30:B34 B36:B40 B42:B46" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
       <formula1>45261</formula1>
     </dataValidation>
   </dataValidations>
@@ -1651,7 +1707,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>A12:E16 A18:E22 A24:E28 A30:E34 A36:E40 A42:E46 A48:E52 A54:E1048576 A1:D3 F1:F3 G4:G10 A11:D11 A17:D17 A23:D23 A29:D29 A35:D35 A41:D41 A47:D47 A53:D53 G54:G1048576 A4:E6 B7:C7 E7 A8:E10</xm:sqref>
+          <xm:sqref>A4:E6 E7 A8:E8 A10:E10 A12:E16 A18:E22 A24:E28 A30:E34 A36:E40 A42:E46 A48:E1048576 A1:D3 F1:F3 G4:G8 B7:C7 A9:D9 A11:D11 A17:D17 A23:D23 A29:D29 A35:D35 A41:D41 A47:D47 G48:G1048576</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="endsWith" priority="11" operator="endsWith" id="{FA4647AC-51FE-4597-AE79-DF1EBCADBA52}">
@@ -1687,7 +1743,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>E4:E10 E12:E16 E18:E22 E24:E28 E30:E34 E36:E40 E42:E46 E48:E52 E54:E1048576</xm:sqref>
+          <xm:sqref>E4:E8 E10 E12:E16 E18:E22 E24:E28 E30:E34 E36:E40 E42:E46 E48:E1048576</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="containsText" priority="8" operator="containsText" id="{FD0F452B-B2F8-4F75-A8CD-A69AC0834E64}">
@@ -1701,10 +1757,24 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>F6:F10</xm:sqref>
+          <xm:sqref>F6:F8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="containsText" priority="7" operator="containsText" id="{88417B48-EA26-4D48-9EFE-B6A1E5C426AE}">
+            <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F10)))</xm:f>
+            <xm:f>Restrictions!$B$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FF00B0F0"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>F10:G10</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="containsText" priority="6" operator="containsText" id="{6407061A-B268-44CE-A52C-133739941B16}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F12)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -1718,7 +1788,7 @@
           <xm:sqref>F12:G16</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="6" operator="containsText" id="{6407061A-B268-44CE-A52C-133739941B16}">
+          <x14:cfRule type="containsText" priority="5" operator="containsText" id="{756A584A-6AAC-4559-9F27-A59B4EFD7F34}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F18)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -1732,7 +1802,7 @@
           <xm:sqref>F18:G22</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="5" operator="containsText" id="{756A584A-6AAC-4559-9F27-A59B4EFD7F34}">
+          <x14:cfRule type="containsText" priority="4" operator="containsText" id="{E988FD75-2909-4816-91C7-1018002A435D}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F24)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -1746,7 +1816,7 @@
           <xm:sqref>F24:G28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="4" operator="containsText" id="{E988FD75-2909-4816-91C7-1018002A435D}">
+          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{D5B6D5DF-9E2A-4C4B-BA82-97D983766AEE}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F30)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -1760,7 +1830,7 @@
           <xm:sqref>F30:G34</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{D5B6D5DF-9E2A-4C4B-BA82-97D983766AEE}">
+          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{1555D56B-E8B5-4F0A-9D80-B2C1016EB105}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F36)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -1774,7 +1844,7 @@
           <xm:sqref>F36:G40</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{1555D56B-E8B5-4F0A-9D80-B2C1016EB105}">
+          <x14:cfRule type="containsText" priority="1" operator="containsText" id="{2F0F41F7-8C93-48A6-B013-C45F8E29AE34}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F42)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -1787,20 +1857,6 @@
           </x14:cfRule>
           <xm:sqref>F42:G46</xm:sqref>
         </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="1" operator="containsText" id="{2F0F41F7-8C93-48A6-B013-C45F8E29AE34}">
-            <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F48)))</xm:f>
-            <xm:f>Restrictions!$B$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FF00B0F0"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>F48:G52</xm:sqref>
-        </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -1809,7 +1865,7 @@
           <x14:formula1>
             <xm:f>Restrictions!$A$1:$D$1</xm:f>
           </x14:formula1>
-          <xm:sqref>E1:E4 E6:E10 E12:E16 E18:E22 E24:E28 E30:E34 E36:E40 E42:E46 E48:E52 E54:E1048576</xm:sqref>
+          <xm:sqref>E1:E4 E6:E8 E10 E12:E16 E18:E22 E24:E28 E30:E34 E36:E40 E42:E46 E48:E1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1842,6 +1898,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a1b10758-7132-46a4-a2fe-7a2cf46f51f4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="f7d9f5a6-831d-4621-8c77-cbcaf993e406" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005A5B8F5EAAC22C48A11F5D9A60E6F21D" ma:contentTypeVersion="16" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="f2b963976306cc54294b7f4545a3c6c4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a1b10758-7132-46a4-a2fe-7a2cf46f51f4" xmlns:ns3="f7d9f5a6-831d-4621-8c77-cbcaf993e406" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e5e135fa2fc1295e1586ddcd9c1a8904" ns2:_="" ns3:_="">
     <xsd:import namespace="a1b10758-7132-46a4-a2fe-7a2cf46f51f4"/>
@@ -2084,27 +2160,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a1b10758-7132-46a4-a2fe-7a2cf46f51f4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="f7d9f5a6-831d-4621-8c77-cbcaf993e406" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0E6F7E92-72FE-4C94-B42F-AE9EA593DE95}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a1b10758-7132-46a4-a2fe-7a2cf46f51f4"/>
+    <ds:schemaRef ds:uri="f7d9f5a6-831d-4621-8c77-cbcaf993e406"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{40597E6F-FA73-4A07-893F-099FDC15B64D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2121,23 +2196,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0E6F7E92-72FE-4C94-B42F-AE9EA593DE95}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="a1b10758-7132-46a4-a2fe-7a2cf46f51f4"/>
-    <ds:schemaRef ds:uri="f7d9f5a6-831d-4621-8c77-cbcaf993e406"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Chore(files): Re-added some documents
</commit_message>
<xml_diff>
--- a/T-CraftMeUp_JonathanJunod.xlsx
+++ b/T-CraftMeUp_JonathanJunod.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pe40boh\Documents\GitHub\Craft-Me-Up\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:11_{49C3D4D1-FA8C-4A30-8C9B-417FD5D42074}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2039DEDB-E2CA-47CA-AD70-10DD1F1CE2F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-75" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
     <sheet name="Restrictions" sheetId="19" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$G$54</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$G$48</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="61">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -186,6 +186,54 @@
   </si>
   <si>
     <t>https://eduvaud-my.sharepoint.com/:u:/r/personal/pb62kjx_eduvaud_ch/_layouts/15/Doc.aspx?sourcedoc=%7B5BF0A89E-E3A6-4CD4-BA7E-BFDC17A68BD3%7D&amp;file=P_CraftMeUp_ClassDiagram.vsdx&amp;fromShare=true&amp;action=default&amp;mobileredirect=true</t>
+  </si>
+  <si>
+    <t>Creating a new version of the classes diagram</t>
+  </si>
+  <si>
+    <t>Debating about the code optimization</t>
+  </si>
+  <si>
+    <t>Debating</t>
+  </si>
+  <si>
+    <t>Github project</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adding a kanban to github </t>
+  </si>
+  <si>
+    <t>Read and complete the CdC written by Neo</t>
+  </si>
+  <si>
+    <t>CdC</t>
+  </si>
+  <si>
+    <t>Coding</t>
+  </si>
+  <si>
+    <t>Correcting the obstacle class</t>
+  </si>
+  <si>
+    <t>https://github.com/users/Jonathan150408/projects/4/views/1</t>
+  </si>
+  <si>
+    <t>Git-problem</t>
+  </si>
+  <si>
+    <t>Solving a problem with the github project issues</t>
+  </si>
+  <si>
+    <t>https://github.com/users/Jonathan150408/projects/6/views/1</t>
+  </si>
+  <si>
+    <t>Updating the classes diagram</t>
+  </si>
+  <si>
+    <t>Correcting Shoot me up</t>
+  </si>
+  <si>
+    <t>Optimizing Shoot me up</t>
   </si>
 </sst>
 </file>
@@ -397,7 +445,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -480,6 +528,14 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="20" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -522,10 +578,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -927,7 +979,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" style="1" customWidth="1"/>
@@ -945,65 +997,65 @@
       <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="32" t="s">
+      <c r="B1" s="34" t="s">
         <v>36</v>
       </c>
-      <c r="C1" s="33"/>
-      <c r="D1" s="30" t="s">
+      <c r="C1" s="35"/>
+      <c r="D1" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="31"/>
-      <c r="F1" s="28" t="s">
+      <c r="E1" s="33"/>
+      <c r="F1" s="30" t="s">
         <v>37</v>
       </c>
-      <c r="G1" s="29"/>
+      <c r="G1" s="31"/>
     </row>
     <row r="2" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="32" t="s">
+      <c r="B2" s="34" t="s">
         <v>35</v>
       </c>
-      <c r="C2" s="33"/>
-      <c r="D2" s="30" t="s">
+      <c r="C2" s="35"/>
+      <c r="D2" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="31"/>
-      <c r="F2" s="28" t="s">
+      <c r="E2" s="33"/>
+      <c r="F2" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="29"/>
+      <c r="G2" s="31"/>
     </row>
     <row r="3" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="32" t="s">
+      <c r="B3" s="34" t="s">
         <v>34</v>
       </c>
-      <c r="C3" s="33"/>
-      <c r="D3" s="30" t="s">
+      <c r="C3" s="35"/>
+      <c r="D3" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="31"/>
-      <c r="F3" s="32" t="s">
+      <c r="E3" s="33"/>
+      <c r="F3" s="34" t="s">
         <v>39</v>
       </c>
-      <c r="G3" s="33"/>
+      <c r="G3" s="35"/>
     </row>
     <row r="4" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="32" t="s">
+      <c r="B4" s="34" t="s">
         <v>38</v>
       </c>
-      <c r="C4" s="36"/>
-      <c r="D4" s="36"/>
-      <c r="E4" s="36"/>
-      <c r="F4" s="36"/>
-      <c r="G4" s="33"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="38"/>
+      <c r="F4" s="38"/>
+      <c r="G4" s="35"/>
     </row>
     <row r="5" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1032,7 +1084,7 @@
       <c r="A6" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="23">
+      <c r="B6" s="25">
         <v>45964</v>
       </c>
       <c r="C6" s="5">
@@ -1044,7 +1096,7 @@
       <c r="E6" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="F6" s="37">
+      <c r="F6" s="24">
         <v>0.59027777777777779</v>
       </c>
       <c r="G6" s="19" t="s">
@@ -1055,7 +1107,7 @@
       <c r="A7" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="B7" s="24"/>
+      <c r="B7" s="26"/>
       <c r="C7" s="7">
         <v>35</v>
       </c>
@@ -1065,16 +1117,16 @@
       <c r="E7" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="F7" s="37">
+      <c r="F7" s="24">
         <v>0.61458333333333337</v>
       </c>
       <c r="G7" s="19"/>
     </row>
-    <row r="8" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="B8" s="24"/>
+      <c r="B8" s="26"/>
       <c r="C8" s="7">
         <v>45</v>
       </c>
@@ -1084,29 +1136,50 @@
       <c r="E8" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="F8" s="37">
+      <c r="F8" s="24">
         <v>0.65625</v>
       </c>
       <c r="G8" s="19" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="6"/>
-      <c r="B9" s="24"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="19"/>
+    <row r="9" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="36">
+        <f>SUM(C6:C8)</f>
+        <v>110</v>
+      </c>
+      <c r="E9" s="36"/>
+      <c r="F9" s="36"/>
+      <c r="G9" s="37"/>
     </row>
     <row r="10" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="9"/>
-      <c r="B10" s="25"/>
-      <c r="C10" s="9"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="7"/>
+      <c r="A10" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" s="23">
+        <v>45970</v>
+      </c>
+      <c r="C10" s="5">
+        <v>30</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="24">
+        <v>0.68055555555555547</v>
+      </c>
       <c r="G10" s="19"/>
     </row>
     <row r="11" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1114,112 +1187,200 @@
         <v>12</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C11" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="34">
-        <f>SUM(C6:C10)</f>
-        <v>110</v>
-      </c>
-      <c r="E11" s="34"/>
-      <c r="F11" s="34"/>
-      <c r="G11" s="35"/>
+      <c r="D11" s="36">
+        <f>SUM(C10:C10)</f>
+        <v>30</v>
+      </c>
+      <c r="E11" s="36"/>
+      <c r="F11" s="36"/>
+      <c r="G11" s="37"/>
     </row>
     <row r="12" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="4"/>
-      <c r="B12" s="23"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="22"/>
+      <c r="A12" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" s="25">
+        <v>45971</v>
+      </c>
+      <c r="C12" s="5">
+        <v>45</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="24">
+        <v>0.57986111111111105</v>
+      </c>
       <c r="G12" s="19"/>
     </row>
     <row r="13" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="6"/>
-      <c r="B13" s="24"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="22"/>
-      <c r="G13" s="19"/>
+      <c r="A13" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B13" s="26"/>
+      <c r="C13" s="7">
+        <v>5</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F13" s="24">
+        <v>0.58680555555555558</v>
+      </c>
+      <c r="G13" s="19" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="14" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="6"/>
-      <c r="B14" s="24"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="7"/>
+      <c r="A14" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B14" s="26"/>
+      <c r="C14" s="7">
+        <v>10</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F14" s="24">
+        <v>0.59375</v>
+      </c>
       <c r="G14" s="19"/>
     </row>
     <row r="15" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="6"/>
-      <c r="B15" s="24"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="7"/>
+      <c r="A15" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B15" s="26"/>
+      <c r="C15" s="7">
+        <v>50</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F15" s="24">
+        <v>0.65625</v>
+      </c>
       <c r="G15" s="19"/>
     </row>
     <row r="16" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="9"/>
-      <c r="B16" s="25"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="19"/>
+      <c r="A16" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B16" s="27"/>
+      <c r="C16" s="9">
+        <v>25</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="F16" s="24">
+        <v>0.61458333333333337</v>
+      </c>
+      <c r="G16" s="19" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="17" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
         <v>12</v>
       </c>
       <c r="B17" s="17" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C17" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="D17" s="34">
+      <c r="D17" s="36">
         <f>SUM(C12:C16)</f>
-        <v>0</v>
-      </c>
-      <c r="E17" s="34"/>
-      <c r="F17" s="34"/>
-      <c r="G17" s="35"/>
+        <v>135</v>
+      </c>
+      <c r="E17" s="36"/>
+      <c r="F17" s="36"/>
+      <c r="G17" s="37"/>
     </row>
     <row r="18" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="4"/>
-      <c r="B18" s="23"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="22"/>
+      <c r="A18" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B18" s="25">
+        <v>45978</v>
+      </c>
+      <c r="C18" s="5">
+        <v>15</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F18" s="24">
+        <v>0.55902777777777779</v>
+      </c>
       <c r="G18" s="19"/>
     </row>
     <row r="19" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="6"/>
-      <c r="B19" s="24"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="22"/>
+      <c r="A19" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B19" s="26"/>
+      <c r="C19" s="7">
+        <v>105</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F19" s="24">
+        <v>0.63888888888888895</v>
+      </c>
       <c r="G19" s="19"/>
     </row>
     <row r="20" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="6"/>
-      <c r="B20" s="24"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="7"/>
+      <c r="A20" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B20" s="26"/>
+      <c r="C20" s="7">
+        <v>25</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F20" s="24">
+        <v>0.64236111111111105</v>
+      </c>
       <c r="G20" s="19"/>
     </row>
     <row r="21" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6"/>
-      <c r="B21" s="24"/>
+      <c r="B21" s="26"/>
       <c r="C21" s="7"/>
       <c r="D21" s="8"/>
       <c r="E21" s="8"/>
@@ -1228,7 +1389,7 @@
     </row>
     <row r="22" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="9"/>
-      <c r="B22" s="25"/>
+      <c r="B22" s="27"/>
       <c r="C22" s="9"/>
       <c r="D22" s="8"/>
       <c r="E22" s="10"/>
@@ -1240,22 +1401,22 @@
         <v>12</v>
       </c>
       <c r="B23" s="17" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C23" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="D23" s="34">
+      <c r="D23" s="36">
         <f>SUM(C18:C22)</f>
-        <v>0</v>
-      </c>
-      <c r="E23" s="34"/>
-      <c r="F23" s="34"/>
-      <c r="G23" s="35"/>
+        <v>145</v>
+      </c>
+      <c r="E23" s="36"/>
+      <c r="F23" s="36"/>
+      <c r="G23" s="37"/>
     </row>
     <row r="24" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4"/>
-      <c r="B24" s="23"/>
+      <c r="B24" s="25"/>
       <c r="C24" s="5"/>
       <c r="D24" s="8"/>
       <c r="E24" s="8"/>
@@ -1264,7 +1425,7 @@
     </row>
     <row r="25" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="6"/>
-      <c r="B25" s="24"/>
+      <c r="B25" s="26"/>
       <c r="C25" s="7"/>
       <c r="D25" s="8"/>
       <c r="E25" s="8"/>
@@ -1273,7 +1434,7 @@
     </row>
     <row r="26" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="6"/>
-      <c r="B26" s="24"/>
+      <c r="B26" s="26"/>
       <c r="C26" s="7"/>
       <c r="D26" s="8"/>
       <c r="E26" s="8"/>
@@ -1282,7 +1443,7 @@
     </row>
     <row r="27" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="6"/>
-      <c r="B27" s="24"/>
+      <c r="B27" s="26"/>
       <c r="C27" s="7"/>
       <c r="D27" s="8"/>
       <c r="E27" s="8"/>
@@ -1291,7 +1452,7 @@
     </row>
     <row r="28" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="9"/>
-      <c r="B28" s="25"/>
+      <c r="B28" s="27"/>
       <c r="C28" s="9"/>
       <c r="D28" s="8"/>
       <c r="E28" s="10"/>
@@ -1303,22 +1464,22 @@
         <v>12</v>
       </c>
       <c r="B29" s="17" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C29" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="D29" s="34">
+      <c r="D29" s="36">
         <f>SUM(C24:C28)</f>
         <v>0</v>
       </c>
-      <c r="E29" s="34"/>
-      <c r="F29" s="34"/>
-      <c r="G29" s="35"/>
+      <c r="E29" s="36"/>
+      <c r="F29" s="36"/>
+      <c r="G29" s="37"/>
     </row>
     <row r="30" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="4"/>
-      <c r="B30" s="23"/>
+      <c r="B30" s="25"/>
       <c r="C30" s="5"/>
       <c r="D30" s="8"/>
       <c r="E30" s="8"/>
@@ -1327,7 +1488,7 @@
     </row>
     <row r="31" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="6"/>
-      <c r="B31" s="24"/>
+      <c r="B31" s="26"/>
       <c r="C31" s="7"/>
       <c r="D31" s="8"/>
       <c r="E31" s="8"/>
@@ -1336,7 +1497,7 @@
     </row>
     <row r="32" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="6"/>
-      <c r="B32" s="24"/>
+      <c r="B32" s="26"/>
       <c r="C32" s="7"/>
       <c r="D32" s="8"/>
       <c r="E32" s="8"/>
@@ -1345,7 +1506,7 @@
     </row>
     <row r="33" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="6"/>
-      <c r="B33" s="24"/>
+      <c r="B33" s="26"/>
       <c r="C33" s="7"/>
       <c r="D33" s="8"/>
       <c r="E33" s="8"/>
@@ -1354,7 +1515,7 @@
     </row>
     <row r="34" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="9"/>
-      <c r="B34" s="25"/>
+      <c r="B34" s="27"/>
       <c r="C34" s="9"/>
       <c r="D34" s="8"/>
       <c r="E34" s="10"/>
@@ -1366,22 +1527,22 @@
         <v>12</v>
       </c>
       <c r="B35" s="17" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C35" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="D35" s="34">
+      <c r="D35" s="36">
         <f>SUM(C30:C34)</f>
         <v>0</v>
       </c>
-      <c r="E35" s="34"/>
-      <c r="F35" s="34"/>
-      <c r="G35" s="35"/>
+      <c r="E35" s="36"/>
+      <c r="F35" s="36"/>
+      <c r="G35" s="37"/>
     </row>
     <row r="36" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="4"/>
-      <c r="B36" s="23"/>
+      <c r="B36" s="25"/>
       <c r="C36" s="5"/>
       <c r="D36" s="8"/>
       <c r="E36" s="8"/>
@@ -1390,7 +1551,7 @@
     </row>
     <row r="37" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="6"/>
-      <c r="B37" s="24"/>
+      <c r="B37" s="26"/>
       <c r="C37" s="7"/>
       <c r="D37" s="8"/>
       <c r="E37" s="8"/>
@@ -1399,7 +1560,7 @@
     </row>
     <row r="38" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="6"/>
-      <c r="B38" s="24"/>
+      <c r="B38" s="26"/>
       <c r="C38" s="7"/>
       <c r="D38" s="8"/>
       <c r="E38" s="8"/>
@@ -1408,7 +1569,7 @@
     </row>
     <row r="39" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="6"/>
-      <c r="B39" s="24"/>
+      <c r="B39" s="26"/>
       <c r="C39" s="7"/>
       <c r="D39" s="8"/>
       <c r="E39" s="8"/>
@@ -1417,7 +1578,7 @@
     </row>
     <row r="40" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="9"/>
-      <c r="B40" s="25"/>
+      <c r="B40" s="27"/>
       <c r="C40" s="9"/>
       <c r="D40" s="8"/>
       <c r="E40" s="10"/>
@@ -1429,22 +1590,22 @@
         <v>12</v>
       </c>
       <c r="B41" s="17" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C41" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="D41" s="34">
+      <c r="D41" s="36">
         <f>SUM(C36:C40)</f>
         <v>0</v>
       </c>
-      <c r="E41" s="34"/>
-      <c r="F41" s="34"/>
-      <c r="G41" s="35"/>
+      <c r="E41" s="36"/>
+      <c r="F41" s="36"/>
+      <c r="G41" s="37"/>
     </row>
     <row r="42" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="4"/>
-      <c r="B42" s="23"/>
+      <c r="B42" s="25"/>
       <c r="C42" s="5"/>
       <c r="D42" s="8"/>
       <c r="E42" s="8"/>
@@ -1453,7 +1614,7 @@
     </row>
     <row r="43" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="6"/>
-      <c r="B43" s="24"/>
+      <c r="B43" s="26"/>
       <c r="C43" s="7"/>
       <c r="D43" s="8"/>
       <c r="E43" s="8"/>
@@ -1462,7 +1623,7 @@
     </row>
     <row r="44" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="6"/>
-      <c r="B44" s="24"/>
+      <c r="B44" s="26"/>
       <c r="C44" s="7"/>
       <c r="D44" s="8"/>
       <c r="E44" s="8"/>
@@ -1471,7 +1632,7 @@
     </row>
     <row r="45" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="6"/>
-      <c r="B45" s="24"/>
+      <c r="B45" s="26"/>
       <c r="C45" s="7"/>
       <c r="D45" s="8"/>
       <c r="E45" s="8"/>
@@ -1480,7 +1641,7 @@
     </row>
     <row r="46" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="9"/>
-      <c r="B46" s="25"/>
+      <c r="B46" s="27"/>
       <c r="C46" s="9"/>
       <c r="D46" s="8"/>
       <c r="E46" s="10"/>
@@ -1492,118 +1653,54 @@
         <v>12</v>
       </c>
       <c r="B47" s="17" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C47" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="D47" s="34">
+      <c r="D47" s="36">
         <f>SUM(C42:C46)</f>
         <v>0</v>
       </c>
-      <c r="E47" s="34"/>
-      <c r="F47" s="34"/>
-      <c r="G47" s="35"/>
-    </row>
-    <row r="48" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="4"/>
-      <c r="B48" s="23"/>
-      <c r="C48" s="5"/>
-      <c r="D48" s="8"/>
-      <c r="E48" s="8"/>
-      <c r="F48" s="22"/>
-      <c r="G48" s="19"/>
-    </row>
-    <row r="49" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="6"/>
-      <c r="B49" s="24"/>
-      <c r="C49" s="7"/>
-      <c r="D49" s="8"/>
-      <c r="E49" s="8"/>
-      <c r="F49" s="22"/>
-      <c r="G49" s="19"/>
-    </row>
-    <row r="50" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="6"/>
-      <c r="B50" s="24"/>
-      <c r="C50" s="7"/>
-      <c r="D50" s="8"/>
-      <c r="E50" s="8"/>
-      <c r="F50" s="7"/>
-      <c r="G50" s="19"/>
-    </row>
-    <row r="51" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="6"/>
-      <c r="B51" s="24"/>
-      <c r="C51" s="7"/>
-      <c r="D51" s="8"/>
-      <c r="E51" s="8"/>
-      <c r="F51" s="7"/>
-      <c r="G51" s="19"/>
-    </row>
-    <row r="52" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="9"/>
-      <c r="B52" s="25"/>
-      <c r="C52" s="9"/>
-      <c r="D52" s="8"/>
-      <c r="E52" s="10"/>
-      <c r="F52" s="7"/>
-      <c r="G52" s="19"/>
-    </row>
-    <row r="53" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B53" s="17" t="s">
-        <v>26</v>
-      </c>
-      <c r="C53" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="D53" s="34">
-        <f>SUM(C48:C52)</f>
-        <v>0</v>
-      </c>
-      <c r="E53" s="34"/>
-      <c r="F53" s="34"/>
-      <c r="G53" s="35"/>
-    </row>
-    <row r="54" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="26" t="s">
+      <c r="E47" s="36"/>
+      <c r="F47" s="36"/>
+      <c r="G47" s="37"/>
+    </row>
+    <row r="48" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="B54" s="27"/>
-      <c r="C54" s="12">
-        <f>MROUND(SUM(C6:C53) /60,0.2)</f>
-        <v>1.8</v>
-      </c>
-      <c r="D54" s="13"/>
-      <c r="E54" s="18"/>
-      <c r="F54" s="20"/>
-      <c r="G54" s="14"/>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" s="15" t="s">
+      <c r="B48" s="29"/>
+      <c r="C48" s="12">
+        <f>MROUND(SUM(C6:C47) /60,0.2)</f>
+        <v>7</v>
+      </c>
+      <c r="D48" s="13"/>
+      <c r="E48" s="18"/>
+      <c r="F48" s="20"/>
+      <c r="G48" s="14"/>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" s="15" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" s="15"/>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" s="15"/>
     </row>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="26">
+    <mergeCell ref="D23:G23"/>
     <mergeCell ref="D29:G29"/>
     <mergeCell ref="D35:G35"/>
     <mergeCell ref="D41:G41"/>
     <mergeCell ref="D47:G47"/>
-    <mergeCell ref="D53:G53"/>
+    <mergeCell ref="D9:G9"/>
     <mergeCell ref="D11:G11"/>
     <mergeCell ref="D17:G17"/>
-    <mergeCell ref="D23:G23"/>
     <mergeCell ref="B4:G4"/>
-    <mergeCell ref="B6:B10"/>
+    <mergeCell ref="B6:B8"/>
     <mergeCell ref="B12:B16"/>
-    <mergeCell ref="B18:B22"/>
     <mergeCell ref="F1:G1"/>
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="D2:E2"/>
@@ -1613,18 +1710,18 @@
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="F3:G3"/>
+    <mergeCell ref="B18:B22"/>
     <mergeCell ref="B24:B28"/>
     <mergeCell ref="B30:B34"/>
+    <mergeCell ref="A48:B48"/>
     <mergeCell ref="B36:B40"/>
-    <mergeCell ref="A54:B54"/>
     <mergeCell ref="B42:B46"/>
-    <mergeCell ref="B48:B52"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C48:C52 C36:C40 C42:C46 C18:C22 B6 C12:C16 C24:C28 C30:C34 C6:C10" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C42:C46 C30:C34 C36:C40 C12:C16 B6 C10 C18:C22 C24:C28 C6:C8" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B12:B16 B18:B22 B24:B28 B30:B34 B36:B40 B42:B46 B48:B52" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B10 B12:B16 B18:B22 B24:B28 B30:B34 B36:B40 B42:B46" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
       <formula1>45261</formula1>
     </dataValidation>
   </dataValidations>
@@ -1651,7 +1748,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>A12:E16 A18:E22 A24:E28 A30:E34 A36:E40 A42:E46 A48:E52 A54:E1048576 A1:D3 F1:F3 G4:G10 A11:D11 A17:D17 A23:D23 A29:D29 A35:D35 A41:D41 A47:D47 A53:D53 G54:G1048576 A4:E6 B7:C7 E7 A8:E10</xm:sqref>
+          <xm:sqref>A4:E6 E7 A8:E8 A10:E10 A12:E16 A24:E28 A30:E34 A36:E40 A42:E46 A48:E1048576 A1:D3 F1:F3 G4:G8 B7:C7 A9:D9 A11:D11 A17:D17 A23:D23 A29:D29 A35:D35 A41:D41 A47:D47 G48:G1048576 A18:E18 A21:E22 A19:C19 A20:D20 E19:E20</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="endsWith" priority="11" operator="endsWith" id="{FA4647AC-51FE-4597-AE79-DF1EBCADBA52}">
@@ -1687,7 +1784,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>E4:E10 E12:E16 E18:E22 E24:E28 E30:E34 E36:E40 E42:E46 E48:E52 E54:E1048576</xm:sqref>
+          <xm:sqref>E4:E8 E10 E12:E16 E18:E22 E24:E28 E30:E34 E36:E40 E42:E46 E48:E1048576</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="containsText" priority="8" operator="containsText" id="{FD0F452B-B2F8-4F75-A8CD-A69AC0834E64}">
@@ -1701,10 +1798,24 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>F6:F10</xm:sqref>
+          <xm:sqref>F6:F8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="containsText" priority="7" operator="containsText" id="{88417B48-EA26-4D48-9EFE-B6A1E5C426AE}">
+            <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F10)))</xm:f>
+            <xm:f>Restrictions!$B$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FF00B0F0"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>F10:G10</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="containsText" priority="6" operator="containsText" id="{6407061A-B268-44CE-A52C-133739941B16}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F12)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -1718,7 +1829,7 @@
           <xm:sqref>F12:G16</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="6" operator="containsText" id="{6407061A-B268-44CE-A52C-133739941B16}">
+          <x14:cfRule type="containsText" priority="5" operator="containsText" id="{756A584A-6AAC-4559-9F27-A59B4EFD7F34}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F18)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -1732,7 +1843,7 @@
           <xm:sqref>F18:G22</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="5" operator="containsText" id="{756A584A-6AAC-4559-9F27-A59B4EFD7F34}">
+          <x14:cfRule type="containsText" priority="4" operator="containsText" id="{E988FD75-2909-4816-91C7-1018002A435D}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F24)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -1746,7 +1857,7 @@
           <xm:sqref>F24:G28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="4" operator="containsText" id="{E988FD75-2909-4816-91C7-1018002A435D}">
+          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{D5B6D5DF-9E2A-4C4B-BA82-97D983766AEE}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F30)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -1760,7 +1871,7 @@
           <xm:sqref>F30:G34</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{D5B6D5DF-9E2A-4C4B-BA82-97D983766AEE}">
+          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{1555D56B-E8B5-4F0A-9D80-B2C1016EB105}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F36)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -1774,7 +1885,7 @@
           <xm:sqref>F36:G40</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{1555D56B-E8B5-4F0A-9D80-B2C1016EB105}">
+          <x14:cfRule type="containsText" priority="1" operator="containsText" id="{2F0F41F7-8C93-48A6-B013-C45F8E29AE34}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F42)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -1787,20 +1898,6 @@
           </x14:cfRule>
           <xm:sqref>F42:G46</xm:sqref>
         </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="1" operator="containsText" id="{2F0F41F7-8C93-48A6-B013-C45F8E29AE34}">
-            <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F48)))</xm:f>
-            <xm:f>Restrictions!$B$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FF00B0F0"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>F48:G52</xm:sqref>
-        </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -1809,7 +1906,7 @@
           <x14:formula1>
             <xm:f>Restrictions!$A$1:$D$1</xm:f>
           </x14:formula1>
-          <xm:sqref>E1:E4 E6:E10 E12:E16 E18:E22 E24:E28 E30:E34 E36:E40 E42:E46 E48:E52 E54:E1048576</xm:sqref>
+          <xm:sqref>E1:E4 E6:E8 E10 E12:E16 E18:E22 E24:E28 E30:E34 E36:E40 E42:E46 E48:E1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>